<commit_message>
Adiciona minuto dos gols na planilha e no site
</commit_message>
<xml_diff>
--- a/dados/dados.xlsx
+++ b/dados/dados.xlsx
@@ -167,7 +167,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gols — um gol do clube por linha: número do Jogo, Autor e Assistencia (deixe vazio se não houve assistência). Para gol contra do adversário, escreva 'Gol contra' em Autor.</t>
+          <t xml:space="preserve">Gols — um gol do clube por linha: número do Jogo, Minuto, Autor e Assistencia (deixe vazio se não houve assistência). Minuto é só o número (ex.: 23); nos acréscimos use 45+2 ou 90+3. Para gol contra do adversário, escreva 'Gol contra' em Autor.</t>
         </is>
       </c>
     </row>
@@ -1217,8 +1217,9 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1229,10 +1230,15 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Minuto</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Autor</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Assistencia</t>
         </is>
@@ -1242,12 +1248,15 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2">
+        <v>12</v>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t xml:space="preserve">Emil Novak</t>
         </is>
@@ -1257,12 +1266,15 @@
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3">
+        <v>55</v>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mateo Ferreira</t>
         </is>
@@ -1272,12 +1284,15 @@
       <c r="A4">
         <v>1</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4">
+        <v>81</v>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t xml:space="preserve">Kenji Sato</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t xml:space="preserve">Yannick Weber</t>
         </is>
@@ -1287,12 +1302,15 @@
       <c r="A5">
         <v>2</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5">
+        <v>34</v>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t xml:space="preserve">Jonas Keller</t>
         </is>
@@ -1302,12 +1320,15 @@
       <c r="A6">
         <v>2</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6">
+        <v>67</v>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t xml:space="preserve">Mateo Ferreira</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t xml:space="preserve">Emil Novak</t>
         </is>
@@ -1317,7 +1338,10 @@
       <c r="A7">
         <v>3</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7">
+        <v>78</v>
+      </c>
+      <c r="C7" t="inlineStr">
         <is>
           <t xml:space="preserve">Emil Novak</t>
         </is>
@@ -1327,12 +1351,15 @@
       <c r="A8">
         <v>4</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8">
+        <v>9</v>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t xml:space="preserve">Emil Novak</t>
         </is>
@@ -1342,12 +1369,15 @@
       <c r="A9">
         <v>4</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9">
+        <v>40</v>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t xml:space="preserve">Jonas Keller</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t xml:space="preserve">Leon Schäfer</t>
         </is>
@@ -1357,12 +1387,15 @@
       <c r="A10">
         <v>4</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10">
+        <v>88</v>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t xml:space="preserve">Mateo Ferreira</t>
         </is>
@@ -1372,12 +1405,15 @@
       <c r="A11">
         <v>6</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11">
+        <v>23</v>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t xml:space="preserve">Mateo Ferreira</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t xml:space="preserve">Emil Novak</t>
         </is>
@@ -1387,12 +1423,15 @@
       <c r="A12">
         <v>6</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12">
+        <v>71</v>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t xml:space="preserve">Niklas Hoffmann</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t xml:space="preserve">Emil Novak</t>
         </is>
@@ -1402,12 +1441,15 @@
       <c r="A13">
         <v>7</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13">
+        <v>63</v>
+      </c>
+      <c r="C13" t="inlineStr">
         <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t xml:space="preserve">Paul Richter</t>
         </is>
@@ -1417,12 +1459,15 @@
       <c r="A14">
         <v>8</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14">
+        <v>18</v>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t xml:space="preserve">Jonas Keller</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>
@@ -1434,6 +1479,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t xml:space="preserve">90+3</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t xml:space="preserve">Gol contra</t>
         </is>
       </c>
@@ -1442,12 +1492,15 @@
       <c r="A16">
         <v>9</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16">
+        <v>52</v>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t xml:space="preserve">Mateo Ferreira</t>
         </is>
@@ -1457,12 +1510,15 @@
       <c r="A17">
         <v>10</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17">
+        <v>7</v>
+      </c>
+      <c r="C17" t="inlineStr">
         <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t xml:space="preserve">Emil Novak</t>
         </is>
@@ -1472,12 +1528,15 @@
       <c r="A18">
         <v>10</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18">
+        <v>29</v>
+      </c>
+      <c r="C18" t="inlineStr">
         <is>
           <t xml:space="preserve">Mateo Ferreira</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t xml:space="preserve">Jonas Keller</t>
         </is>
@@ -1489,6 +1548,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t xml:space="preserve">45+1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>
       </c>
@@ -1497,12 +1561,15 @@
       <c r="A20">
         <v>10</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20">
+        <v>84</v>
+      </c>
+      <c r="C20" t="inlineStr">
         <is>
           <t xml:space="preserve">Kenji Sato</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>
@@ -1512,12 +1579,15 @@
       <c r="A21">
         <v>11</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21">
+        <v>15</v>
+      </c>
+      <c r="C21" t="inlineStr">
         <is>
           <t xml:space="preserve">Emil Novak</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t xml:space="preserve">Felix Wagner</t>
         </is>
@@ -1527,12 +1597,15 @@
       <c r="A22">
         <v>11</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22">
+        <v>60</v>
+      </c>
+      <c r="C22" t="inlineStr">
         <is>
           <t xml:space="preserve">Mateo Ferreira</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>
@@ -1542,12 +1615,15 @@
       <c r="A23">
         <v>12</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23">
+        <v>38</v>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t xml:space="preserve">Jonas Keller</t>
         </is>
@@ -1557,12 +1633,15 @@
       <c r="A24">
         <v>12</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24">
+        <v>74</v>
+      </c>
+      <c r="C24" t="inlineStr">
         <is>
           <t xml:space="preserve">Felix Wagner</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t xml:space="preserve">Emil Novak</t>
         </is>
@@ -1572,12 +1651,15 @@
       <c r="A25">
         <v>12</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25">
+        <v>89</v>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t xml:space="preserve">Mateo Ferreira</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t xml:space="preserve">Lukas Brandt</t>
         </is>

</xml_diff>

<commit_message>
Busca título, data e thumb dos episódios no canal do YouTube
</commit_message>
<xml_diff>
--- a/dados/dados.xlsx
+++ b/dados/dados.xlsx
@@ -153,7 +153,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Episodios — um episódio por linha: número, temporada, título, data de lançamento, link do vídeo e um resumo curto.</t>
+          <t xml:space="preserve">Episodios — um episódio por linha: número, temporada e um resumo curto. Titulo, Data e Link YouTube podem ficar em branco: o site busca sozinho no canal (vídeos com 'EP 01', 'EP 02'... no título). Se preencher, o que estiver na planilha tem prioridade.</t>
         </is>
       </c>
     </row>
@@ -568,16 +568,6 @@
           <t xml:space="preserve">2026/27</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">O recomeço: Wolfsburg na 2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15/09/2026</t>
-        </is>
-      </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Estreia da carreira: vitória fora de casa na Copa e começo de liga invicto, com Brandt já decidindo.</t>
@@ -593,16 +583,6 @@
           <t xml:space="preserve">2026/27</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Primeira derrota em Gelsenkirchen</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22/09/2026</t>
-        </is>
-      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Goleada sobre o Karlsruhe em casa, mas o Schalke encerrou a invencibilidade na liga.</t>
@@ -618,16 +598,6 @@
           <t xml:space="preserve">2026/27</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Adeus à Copa</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">29/09/2026</t>
-        </is>
-      </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Vitória sobre o Paderborn, eliminação para o Werder Bremen na DFB-Pokal e empate dramático em Hannover.</t>
@@ -643,16 +613,6 @@
           <t xml:space="preserve">2026/27</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Goleada em Darmstadt</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">06/10/2026</t>
-        </is>
-      </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Vitória magra contra o Nürnberg e 4 a 0 fora de casa para entrar de vez na briga pelo acesso.</t>
@@ -666,16 +626,6 @@
       <c r="B6" t="inlineStr">
         <is>
           <t xml:space="preserve">2026/27</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quatro seguidas e a briga pelo acesso</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">13/10/2026</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dados da planilha e do YouTube
</commit_message>
<xml_diff>
--- a/dados/dados.xlsx
+++ b/dados/dados.xlsx
@@ -39,111 +39,114 @@
     <t>2. Preencha a partir da linha 2. Uma linha = um registro. Listas suspensas ajudam nas colunas Local, Competicao, Posicao, Status e Confirmado.</t>
   </si>
   <si>
+    <t>3. Depois de salvar, o site atualiza sozinho (ou envie o arquivo para a pasta 'dados' do site no GitHub com o nome dados.xlsx).</t>
+  </si>
+  <si>
+    <t>ABAS</t>
+  </si>
+  <si>
     <t>Episodio</t>
   </si>
   <si>
-    <t>3. Depois de salvar, o site atualiza sozinho (ou envie o arquivo para a pasta 'dados' do site no GitHub com o nome dados.xlsx).</t>
-  </si>
-  <si>
-    <t>ABAS</t>
+    <t>Clube — configurações gerais: nome do portal, cores, temporada atual e zonas da tabela (acesso, playoff, rebaixamento).</t>
+  </si>
+  <si>
+    <t>Episodios — um episódio por linha: número, temporada e um resumo curto. Titulo, Data e Link YouTube podem ficar em branco: o site busca sozinho no canal (vídeos com 'EP 01', 'EP 02'... no título). Se preencher, o que estiver na planilha tem prioridade. A INTRO entra sozinha pelo YouTube.</t>
+  </si>
+  <si>
+    <t>Jogos — um jogo por linha, em ordem cronológica. A coluna Jogo é um número sequencial (1, 2, 3...) e é ela que liga os gols ao jogo. O resultado (V/E/D) é calculado pelo site.</t>
+  </si>
+  <si>
+    <t>Gols — um gol do clube por linha: número do Jogo, Minuto, Autor e Assistencia (deixe vazio se não houve assistência). Minuto é só o número (ex.: 23); nos acréscimos use 45+2 ou 90+3. Para gol contra do adversário, escreva 'Gol contra' em Autor.</t>
+  </si>
+  <si>
+    <t>Classificacao — a tabela completa ao final de cada episódio (todas as 18 equipes, uma linha cada). Pontos e saldo de gols são calculados pelo site.</t>
+  </si>
+  <si>
+    <t>Elenco — jogadores do elenco com posição e número. Use exatamente os mesmos nomes da aba Gols.</t>
+  </si>
+  <si>
+    <t>Recordes — recordes reais do clube até o início da série (temporada 2026/27). NÃO altere a coluna Chave. Edite Valor, Detentor e Quando. Confirmado = SIM tira o aviso 'a confirmar' do site.</t>
+  </si>
+  <si>
+    <t>Metas — objetivos da carreira, com Status: Em andamento, Concluída ou Falhou.</t>
+  </si>
+  <si>
+    <t>Titulos — títulos conquistados na carreira (uma linha por título).</t>
+  </si>
+  <si>
+    <t>EXEMPLOS DE PREENCHIMENTO</t>
+  </si>
+  <si>
+    <t>Episodios:  1 | 2026/27 | (vazio) | (vazio) | (vazio) | Estreia na 2. Bundesliga com vitória em casa.</t>
+  </si>
+  <si>
+    <t>Chave</t>
+  </si>
+  <si>
+    <t>Jogos:  1 | 1 | 2026/27 | 2. Bundesliga | 1 | Hertha BSC | Casa | 2 | 0</t>
+  </si>
+  <si>
+    <t>Temporada</t>
   </si>
   <si>
     <t>Jogo</t>
   </si>
   <si>
-    <t>Chave</t>
-  </si>
-  <si>
-    <t>Clube — configurações gerais: nome do portal, cores, temporada atual e zonas da tabela (acesso, playoff, rebaixamento).</t>
-  </si>
-  <si>
-    <t>Episodios — um episódio por linha: número, temporada e um resumo curto. Titulo, Data e Link YouTube podem ficar em branco: o site busca sozinho no canal (vídeos com 'EP 01', 'EP 02'... no título). Se preencher, o que estiver na planilha tem prioridade. A INTRO entra sozinha pelo YouTube.</t>
-  </si>
-  <si>
-    <t>Jogos — um jogo por linha, em ordem cronológica. A coluna Jogo é um número sequencial (1, 2, 3...) e é ela que liga os gols ao jogo. O resultado (V/E/D) é calculado pelo site.</t>
-  </si>
-  <si>
-    <t>Gols — um gol do clube por linha: número do Jogo, Minuto, Autor e Assistencia (deixe vazio se não houve assistência). Minuto é só o número (ex.: 23); nos acréscimos use 45+2 ou 90+3. Para gol contra do adversário, escreva 'Gol contra' em Autor.</t>
-  </si>
-  <si>
-    <t>Classificacao — a tabela completa ao final de cada episódio (todas as 18 equipes, uma linha cada). Pontos e saldo de gols são calculados pelo site.</t>
-  </si>
-  <si>
-    <t>Elenco — jogadores do elenco com posição e número. Use exatamente os mesmos nomes da aba Gols.</t>
-  </si>
-  <si>
-    <t>Temporada</t>
-  </si>
-  <si>
-    <t>Recordes — recordes reais do clube até o início da série (temporada 2026/27). NÃO altere a coluna Chave. Edite Valor, Detentor e Quando. Confirmado = SIM tira o aviso 'a confirmar' do site.</t>
-  </si>
-  <si>
     <t>Titulo</t>
   </si>
   <si>
-    <t>Metas — objetivos da carreira, com Status: Em andamento, Concluída ou Falhou.</t>
+    <t>Gols:  1 | 34 | Nome do Jogador | Nome de quem deu a assistência</t>
   </si>
   <si>
     <t>Valor</t>
   </si>
   <si>
-    <t>Titulos — títulos conquistados na carreira (uma linha por título).</t>
-  </si>
-  <si>
     <t>Data</t>
   </si>
   <si>
+    <t>Classificacao:  1 | 1 | VfL Wolfsburg | 1 | 1 | 0 | 0 | 2 | 0   (Episodio | Posicao | Time | J | V | E | D | GP | GC)</t>
+  </si>
+  <si>
     <t>Descricao</t>
   </si>
   <si>
-    <t>EXEMPLOS DE PREENCHIMENTO</t>
+    <t>Elenco:  Nome do Jogador | ATA | 9 | Alemanha</t>
   </si>
   <si>
     <t>Link YouTube</t>
   </si>
   <si>
+    <t>Resumo</t>
+  </si>
+  <si>
+    <t>ATENÇÃO: os recordes reais estão marcados como 'a confirmar'. Confira cada valor antes de divulgar e mude Confirmado para SIM.</t>
+  </si>
+  <si>
+    <t>nome_portal</t>
+  </si>
+  <si>
     <t>Competicao</t>
   </si>
   <si>
-    <t>Episodios:  1 | 2026/27 | (vazio) | (vazio) | (vazio) | Estreia na 2. Bundesliga com vitória em casa.</t>
-  </si>
-  <si>
-    <t>Resumo</t>
-  </si>
-  <si>
-    <t>nome_portal</t>
-  </si>
-  <si>
     <t>Rodada</t>
   </si>
   <si>
-    <t>Jogos:  1 | 1 | 2026/27 | 2. Bundesliga | 1 | Hertha BSC | Casa | 2 | 0</t>
-  </si>
-  <si>
-    <t>Gols:  1 | 34 | Nome do Jogador | Nome de quem deu a assistência</t>
-  </si>
-  <si>
     <t>Adversario</t>
   </si>
   <si>
-    <t>Classificacao:  1 | 1 | VfL Wolfsburg | 1 | 1 | 0 | 0 | 2 | 0   (Episodio | Posicao | Time | J | V | E | D | GP | GC)</t>
-  </si>
-  <si>
     <t>Local</t>
   </si>
   <si>
-    <t>Elenco:  Nome do Jogador | ATA | 9 | Alemanha</t>
-  </si>
-  <si>
     <t>Gols Pro</t>
   </si>
   <si>
+    <t>2026/27</t>
+  </si>
+  <si>
     <t>Histórias em Campo</t>
   </si>
   <si>
-    <t>2026/27</t>
-  </si>
-  <si>
     <t>Gols Contra</t>
   </si>
   <si>
@@ -159,21 +162,21 @@
     <t>VfL Wolfsburg</t>
   </si>
   <si>
+    <t>26/27</t>
+  </si>
+  <si>
     <t>Nome do clube exatamente como aparece na aba Classificacao</t>
   </si>
   <si>
-    <t>ATENÇÃO: os recordes reais estão marcados como 'a confirmar'. Confira cada valor antes de divulgar e mude Confirmado para SIM.</t>
-  </si>
-  <si>
-    <t>26/27</t>
-  </si>
-  <si>
     <t>canal</t>
   </si>
   <si>
     <t>@gabbiDOMFC</t>
   </si>
   <si>
+    <t>https://www.youtube.com/watch?v=AMmtV3qhNEI</t>
+  </si>
+  <si>
     <t>Nome do canal</t>
   </si>
   <si>
@@ -183,66 +186,63 @@
     <t>https://www.youtube.com/@gabbiDOMFC</t>
   </si>
   <si>
-    <t>https://www.youtube.com/watch?v=AMmtV3qhNEI</t>
-  </si>
-  <si>
     <t>Link do canal no YouTube</t>
   </si>
   <si>
     <t>temporada_atual</t>
   </si>
   <si>
+    <t>Temporada mostrada na página inicial</t>
+  </si>
+  <si>
+    <t>competicao_liga</t>
+  </si>
+  <si>
+    <t>2. Bundesliga</t>
+  </si>
+  <si>
+    <t>Nome da liga, igual ao usado na aba Jogos</t>
+  </si>
+  <si>
+    <t>cor_primaria</t>
+  </si>
+  <si>
+    <t>#65B32E</t>
+  </si>
+  <si>
+    <t>Cor principal do site (código hexadecimal)</t>
+  </si>
+  <si>
+    <t>cor_secundaria</t>
+  </si>
+  <si>
+    <t>#1E4D2B</t>
+  </si>
+  <si>
+    <t>Cor de apoio (fundo do topo)</t>
+  </si>
+  <si>
+    <t>escudo</t>
+  </si>
+  <si>
     <t>DFB-Pokal</t>
   </si>
   <si>
-    <t>Temporada mostrada na página inicial</t>
-  </si>
-  <si>
-    <t>competicao_liga</t>
+    <t>Nome do arquivo de imagem do escudo colocado na pasta do site (ex.: escudo.png). Vazio = monograma</t>
   </si>
   <si>
     <t>1. FC Kaiserslautern</t>
   </si>
   <si>
-    <t>2. Bundesliga</t>
-  </si>
-  <si>
-    <t>Nome da liga, igual ao usado na aba Jogos</t>
-  </si>
-  <si>
-    <t>cor_primaria</t>
-  </si>
-  <si>
-    <t>#65B32E</t>
-  </si>
-  <si>
-    <t>Cor principal do site (código hexadecimal)</t>
+    <t>zona_acesso</t>
+  </si>
+  <si>
+    <t>Até esta posição: acesso direto</t>
   </si>
   <si>
     <t>Casa</t>
   </si>
   <si>
-    <t>cor_secundaria</t>
-  </si>
-  <si>
-    <t>#1E4D2B</t>
-  </si>
-  <si>
-    <t>Cor de apoio (fundo do topo)</t>
-  </si>
-  <si>
-    <t>escudo</t>
-  </si>
-  <si>
-    <t>Nome do arquivo de imagem do escudo colocado na pasta do site (ex.: escudo.png). Vazio = monograma</t>
-  </si>
-  <si>
-    <t>zona_acesso</t>
-  </si>
-  <si>
-    <t>Até esta posição: acesso direto</t>
-  </si>
-  <si>
     <t>zona_playoff_acesso</t>
   </si>
   <si>
@@ -258,6 +258,9 @@
     <t>zona_rebaixamento</t>
   </si>
   <si>
+    <t>Início eletrizante do modo carreira realista com o Wolfsburg agora no comando de um antigo conhecido: Andrés D'Alessandro. Um esboço de time já apresenta gratas surpresas para o decorrer da temporada.</t>
+  </si>
+  <si>
     <t>A partir desta posição: rebaixamento direto</t>
   </si>
   <si>
@@ -270,22 +273,28 @@
     <t>SIM mostra um aviso de dados de exemplo no site</t>
   </si>
   <si>
+    <t>SÓ TEM RETRANQUEIRO NA SEGUNDA DIVISÃO? | FC 27 Modo Carreira Realista Wolfsburg| EP 02</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=eB3sg-pBc1k</t>
+  </si>
+  <si>
     <t>Hannover 96</t>
   </si>
   <si>
     <t>Fora</t>
   </si>
   <si>
-    <t>Início eletrizante do modo carreira realista com o Wolfsburg agora no comando de um antigo conhecido: Andrés D'Alessandro. Um esboço de time já apresenta gratas surpresas para o decorrer da temporada.</t>
-  </si>
-  <si>
     <t>Karlsruher SC</t>
   </si>
   <si>
-    <t>SÓ TEM RETRANQUEIRO NA SEGUNDA DIVISÃO? | FC 27 Modo Carreira Realista Wolfsburg| EP 02</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=eB3sg-pBc1k</t>
+    <t>D'Alessandro está com dificuldades de enfrentar clubes que acabam joganado de forma mais defensiva. Será que ele consegue encontrar uma solução para furar essas retrancas? Descubra neste episódio.</t>
+  </si>
+  <si>
+    <t>TEMOS um CRISTIANO RONALDO JAPONÊS?! 🐐 | FC 27 Modo Carreira Realista Wolfsburg| EP 03</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=mJnFU4fK3lQ</t>
   </si>
   <si>
     <t>Fußball-Club Energie Cottbus</t>
@@ -294,13 +303,13 @@
     <t>FC St. Pauli</t>
   </si>
   <si>
-    <t>D'Alessandro está com dificuldades de enfrentar clubes que acabam joganado de forma mais defensiva. Será que ele consegue encontrar uma solução para furar essas retrancas? Descubra neste episódio.</t>
-  </si>
-  <si>
-    <t>TEMOS um CRISTIANO RONALDO JAPONÊS?! 🐐 | FC 27 Modo Carreira Realista Wolfsburg| EP 03</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=mJnFU4fK3lQ</t>
+    <t xml:space="preserve">A sensação japonesa não se cansa de marcar. Será que estamos diante de um CR7 nipônico? </t>
+  </si>
+  <si>
+    <t>O nível SUBIU! Tomamos um AMASSO? | FC 27 Modo Carreira Realista Wolfsburg| EP 04</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=LW1zoO_I704</t>
   </si>
   <si>
     <t>SV Darmstadt 98</t>
@@ -309,16 +318,16 @@
     <t>1. FC Nürnberg</t>
   </si>
   <si>
-    <t xml:space="preserve">A sensação japonesa não se cansa de marcar. Será que estamos diante de um CR7 nipônico? </t>
+    <t>Os sliders chegaram com tudo, a dificuldade aumentou e nosso time sentiu na pele. Será o fim da boa fase?</t>
   </si>
   <si>
     <t>1. Fußballclub Heidenheim 1846</t>
   </si>
   <si>
-    <t>O nível SUBIU! Tomamos um AMASSO? | FC 27 Modo Carreira Realista Wolfsburg| EP 04</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=LW1zoO_I704</t>
+    <t>ELE está nos salvando do PIOR! | FC 27 Modo Carreira Realista Wolfsburg| EP 05</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=hc248ZsuHh8</t>
   </si>
   <si>
     <t>VfL Bochum</t>
@@ -327,22 +336,13 @@
     <t>Sport-Club Freiburg</t>
   </si>
   <si>
-    <t>Os sliders chegaram com tudo, a dificuldade aumentou e nosso time sentiu na pele. Será o fim da boa fase?</t>
-  </si>
-  <si>
-    <t>ELE está nos salvando do PIOR! | FC 27 Modo Carreira Realista Wolfsburg| EP 05</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=hc248ZsuHh8</t>
+    <t>Com os adversários cada vez mais complicados apenas um homem pode nos salvar... Descubra no episódio neste episódio!</t>
   </si>
   <si>
     <t>Verein für Leibesübungen von 1899</t>
   </si>
   <si>
     <t>Hertha BSC</t>
-  </si>
-  <si>
-    <t>Com os adversários cada vez mais complicados apenas um homem pode nos salvar... Descubra no episódio neste episódio!</t>
   </si>
   <si>
     <t xml:space="preserve">Kieler Sportvereinigung Holstein von 1900 e.V.
@@ -533,70 +533,139 @@
     <t>Grzywacz</t>
   </si>
   <si>
+    <t>Recorde</t>
+  </si>
+  <si>
+    <t>Detentor</t>
+  </si>
+  <si>
+    <t>Quando</t>
+  </si>
+  <si>
+    <t>Observacao</t>
+  </si>
+  <si>
+    <t>Confirmado</t>
+  </si>
+  <si>
+    <t>seq_vitorias</t>
+  </si>
+  <si>
     <t>MC</t>
   </si>
   <si>
+    <t>Maior sequência de vitórias</t>
+  </si>
+  <si>
     <t>Suécia</t>
   </si>
   <si>
+    <t>Bundesliga 2008/09</t>
+  </si>
+  <si>
+    <t>Sequência da campanha do título alemão</t>
+  </si>
+  <si>
     <t>Gerhardt</t>
   </si>
   <si>
+    <t>invencibilidade</t>
+  </si>
+  <si>
     <t>Kosovo</t>
   </si>
   <si>
+    <t>Maior série invicta</t>
+  </si>
+  <si>
+    <t>Preencha com o recorde real do clube</t>
+  </si>
+  <si>
     <t>Vranckx</t>
   </si>
   <si>
+    <t>maior_goleada</t>
+  </si>
+  <si>
     <t>Bélgica</t>
   </si>
   <si>
+    <t>Maior goleada (saldo de gols)</t>
+  </si>
+  <si>
+    <t>Valor = saldo de gols. Use Quando para o placar e o adversário</t>
+  </si>
+  <si>
     <t>Hensel</t>
   </si>
   <si>
+    <t>gols_temporada</t>
+  </si>
+  <si>
+    <t>Mais gols de um jogador numa temporada</t>
+  </si>
+  <si>
+    <t>Grafite</t>
+  </si>
+  <si>
     <t>Dárdai</t>
   </si>
   <si>
+    <t>Artilheiro da Bundesliga na temporada do título</t>
+  </si>
+  <si>
     <t>MEI</t>
   </si>
   <si>
     <t>Hungria</t>
   </si>
   <si>
-    <t>Recorde</t>
+    <t>assist_temporada</t>
+  </si>
+  <si>
+    <t>Mais assistências numa temporada</t>
+  </si>
+  <si>
+    <t>Kevin De Bruyne</t>
+  </si>
+  <si>
+    <t>Bundesliga 2014/15</t>
+  </si>
+  <si>
+    <t>artilheiro_historico</t>
+  </si>
+  <si>
+    <t>Maior artilheiro da história do clube</t>
   </si>
   <si>
     <t>ATA</t>
   </si>
   <si>
-    <t>Detentor</t>
-  </si>
-  <si>
-    <t>Quando</t>
-  </si>
-  <si>
-    <t>Observacao</t>
-  </si>
-  <si>
-    <t>Confirmado</t>
-  </si>
-  <si>
-    <t>seq_vitorias</t>
-  </si>
-  <si>
-    <t>Maior sequência de vitórias</t>
+    <t>Edin Džeko</t>
+  </si>
+  <si>
+    <t>2007–2011</t>
+  </si>
+  <si>
+    <t>Gols na Bundesliga</t>
+  </si>
+  <si>
+    <t>titulos</t>
   </si>
   <si>
     <t>Benedict</t>
   </si>
   <si>
+    <t>Títulos de expressão</t>
+  </si>
+  <si>
     <t>PE</t>
   </si>
   <si>
-    <t>Bundesliga 2008/09</t>
-  </si>
-  <si>
-    <t>Sequência da campanha do título alemão</t>
+    <t>2009–2015</t>
+  </si>
+  <si>
+    <t>Bundesliga 2008/09 · DFB-Pokal 2014/15 · Supercopa da Alemanha 2015</t>
   </si>
   <si>
     <t>Amoura</t>
@@ -608,91 +677,22 @@
     <t>Hornby</t>
   </si>
   <si>
-    <t>invencibilidade</t>
-  </si>
-  <si>
     <t>Escócia</t>
   </si>
   <si>
-    <t>Maior série invicta</t>
-  </si>
-  <si>
-    <t>Preencha com o recorde real do clube</t>
-  </si>
-  <si>
     <t>Glatzel</t>
   </si>
   <si>
-    <t>maior_goleada</t>
-  </si>
-  <si>
-    <t>Maior goleada (saldo de gols)</t>
-  </si>
-  <si>
-    <t>Valor = saldo de gols. Use Quando para o placar e o adversário</t>
-  </si>
-  <si>
     <t>Japão</t>
   </si>
   <si>
-    <t>gols_temporada</t>
-  </si>
-  <si>
-    <t>Mais gols de um jogador numa temporada</t>
-  </si>
-  <si>
     <t>Besio</t>
   </si>
   <si>
-    <t>Grafite</t>
-  </si>
-  <si>
-    <t>Artilheiro da Bundesliga na temporada do título</t>
-  </si>
-  <si>
     <t>Suíça</t>
   </si>
   <si>
-    <t>assist_temporada</t>
-  </si>
-  <si>
-    <t>Mais assistências numa temporada</t>
-  </si>
-  <si>
-    <t>Kevin De Bruyne</t>
-  </si>
-  <si>
-    <t>Bundesliga 2014/15</t>
-  </si>
-  <si>
     <t>Base</t>
-  </si>
-  <si>
-    <t>artilheiro_historico</t>
-  </si>
-  <si>
-    <t>Maior artilheiro da história do clube</t>
-  </si>
-  <si>
-    <t>Edin Džeko</t>
-  </si>
-  <si>
-    <t>2007–2011</t>
-  </si>
-  <si>
-    <t>Gols na Bundesliga</t>
-  </si>
-  <si>
-    <t>titulos</t>
-  </si>
-  <si>
-    <t>Títulos de expressão</t>
-  </si>
-  <si>
-    <t>2009–2015</t>
-  </si>
-  <si>
-    <t>Bundesliga 2008/09 · DFB-Pokal 2014/15 · Supercopa da Alemanha 2015</t>
   </si>
   <si>
     <t>Meta</t>
@@ -1102,7 +1102,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -1110,52 +1110,52 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18">
@@ -1163,32 +1163,32 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
@@ -1196,7 +1196,7 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1"/>
@@ -2196,13 +2196,13 @@
   <sheetData>
     <row r="1" ht="19.5" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -3208,35 +3208,35 @@
   <sheetData>
     <row r="1" ht="19.5" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4">
@@ -3247,15 +3247,15 @@
         <v>48</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>53</v>
@@ -3269,59 +3269,59 @@
         <v>38</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>59</v>
-      </c>
       <c r="C7" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B11" s="5">
         <v>2.0</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12">
@@ -3354,18 +3354,18 @@
         <v>17.0</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -4374,22 +4374,22 @@
   <sheetData>
     <row r="1" ht="19.5" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2">
@@ -4400,16 +4400,16 @@
         <v>38</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D2" s="7">
         <v>46302.0</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3">
@@ -4420,16 +4420,16 @@
         <v>38</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D3" s="7">
         <v>46304.0</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4">
@@ -4440,16 +4440,16 @@
         <v>38</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D4" s="7">
         <v>46308.0</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5">
@@ -4460,16 +4460,16 @@
         <v>38</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D5" s="7">
         <v>46311.0</v>
       </c>
       <c r="E5" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="F5" s="9" t="s">
         <v>97</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="6">
@@ -4480,16 +4480,16 @@
         <v>38</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D6" s="7">
         <v>46315.0</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -5508,31 +5508,31 @@
   <sheetData>
     <row r="1" ht="19.5" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2">
@@ -5543,19 +5543,19 @@
         <v>1.0</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="E2" s="6">
         <v>1.0</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H2" s="6">
         <v>4.0</v>
@@ -5572,19 +5572,19 @@
         <v>1.0</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E3" s="6">
         <v>1.0</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H3" s="6">
         <v>4.0</v>
@@ -5601,19 +5601,19 @@
         <v>1.0</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E4" s="6">
         <v>2.0</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H4" s="6">
         <v>2.0</v>
@@ -5630,19 +5630,19 @@
         <v>1.0</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E5" s="6">
         <v>3.0</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H5" s="6">
         <v>2.0</v>
@@ -5659,19 +5659,19 @@
         <v>2.0</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E6" s="6">
         <v>4.0</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H6" s="6">
         <v>2.0</v>
@@ -5688,19 +5688,19 @@
         <v>2.0</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E7" s="6">
         <v>5.0</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H7" s="6">
         <v>0.0</v>
@@ -5717,19 +5717,19 @@
         <v>2.0</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E8" s="6">
         <v>6.0</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H8" s="6">
         <v>1.0</v>
@@ -5746,19 +5746,19 @@
         <v>2.0</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E9" s="6">
         <v>7.0</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H9" s="6">
         <v>1.0</v>
@@ -5775,19 +5775,19 @@
         <v>3.0</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E10" s="6">
         <v>8.0</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H10" s="6">
         <v>4.0</v>
@@ -5804,19 +5804,19 @@
         <v>3.0</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E11" s="6">
         <v>9.0</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H11" s="6">
         <v>1.0</v>
@@ -5833,19 +5833,19 @@
         <v>3.0</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="E12" s="6">
         <v>2.0</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H12" s="6">
         <v>0.0</v>
@@ -5862,19 +5862,19 @@
         <v>3.0</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E13" s="6">
         <v>10.0</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H13" s="6">
         <v>5.0</v>
@@ -5891,19 +5891,19 @@
         <v>4.0</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E14" s="6">
         <v>11.0</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H14" s="6">
         <v>3.0</v>
@@ -5920,10 +5920,10 @@
         <v>4.0</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E15" s="6">
         <v>12.0</v>
@@ -5932,7 +5932,7 @@
         <v>106</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H15" s="6">
         <v>1.0</v>
@@ -5949,10 +5949,10 @@
         <v>4.0</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E16" s="6">
         <v>13.0</v>
@@ -5961,7 +5961,7 @@
         <v>107</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H16" s="6">
         <v>1.0</v>
@@ -5978,10 +5978,10 @@
         <v>5.0</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E17" s="6">
         <v>14.0</v>
@@ -5990,7 +5990,7 @@
         <v>108</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H17" s="6">
         <v>1.0</v>
@@ -6007,10 +6007,10 @@
         <v>5.0</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E18" s="6">
         <v>15.0</v>
@@ -6019,7 +6019,7 @@
         <v>109</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H18" s="6">
         <v>2.0</v>
@@ -6036,10 +6036,10 @@
         <v>5.0</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E19" s="6">
         <v>16.0</v>
@@ -6048,7 +6048,7 @@
         <v>110</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H19" s="6">
         <v>2.0</v>
@@ -10012,7 +10012,7 @@
   <sheetData>
     <row r="1" ht="19.5" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>111</v>
@@ -11509,7 +11509,7 @@
   <sheetData>
     <row r="1" ht="19.5" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>124</v>
@@ -12536,7 +12536,7 @@
     <col customWidth="1" min="3" max="3" width="9.0"/>
     <col customWidth="1" min="4" max="4" width="16.0"/>
     <col customWidth="1" min="5" max="5" width="10.75"/>
-    <col customWidth="1" min="6" max="6" width="7.75"/>
+    <col customWidth="1" min="6" max="6" width="9.38"/>
     <col customWidth="1" min="7" max="26" width="8.63"/>
   </cols>
   <sheetData>
@@ -12820,10 +12820,10 @@
         <v>119</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>141</v>
@@ -12831,10 +12831,10 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="6" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>143</v>
@@ -12848,10 +12848,10 @@
         <v>120</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>141</v>
@@ -12859,13 +12859,13 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="6" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>141</v>
@@ -12873,10 +12873,10 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>174</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>168</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>143</v>
@@ -12887,13 +12887,13 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="6" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>177</v>
+        <v>196</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>141</v>
@@ -12904,7 +12904,7 @@
         <v>114</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>143</v>
@@ -12918,7 +12918,7 @@
         <v>117</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>143</v>
@@ -12932,10 +12932,10 @@
         <v>118</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>141</v>
@@ -12943,10 +12943,10 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="6" t="s">
-        <v>186</v>
+        <v>208</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>187</v>
+        <v>210</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>143</v>
@@ -12957,13 +12957,13 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="6" t="s">
-        <v>190</v>
+        <v>213</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>191</v>
+        <v>214</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>141</v>
@@ -12971,13 +12971,13 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="6" t="s">
-        <v>192</v>
+        <v>215</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="E31" s="6" t="s">
         <v>141</v>
@@ -12985,10 +12985,10 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="6" t="s">
-        <v>197</v>
+        <v>217</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>143</v>
@@ -13002,10 +13002,10 @@
         <v>115</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>141</v>
@@ -13013,13 +13013,13 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="6" t="s">
-        <v>204</v>
+        <v>219</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>141</v>
@@ -13030,13 +13030,13 @@
         <v>122</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>143</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="F35" s="7">
         <v>46296.0</v>
@@ -14366,166 +14366,166 @@
   <sheetData>
     <row r="1" ht="19.5" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="C2" s="5">
         <v>10.0</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>196</v>
+        <v>183</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>198</v>
+        <v>185</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="C5" s="5">
         <v>28.0</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>205</v>
+        <v>192</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="C6" s="5">
         <v>20.0</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="C7" s="5">
         <v>66.0</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="C8" s="5">
         <v>3.0</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9">
@@ -15738,7 +15738,7 @@
         <v>223</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2">

</xml_diff>